<commit_message>
Neutral smoke workbook; fix stale evaluator references; clarify GT alias map
</commit_message>
<xml_diff>
--- a/samples/test_smoke.xlsx
+++ b/samples/test_smoke.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="entities" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="urls" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="questions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="config" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="entities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="urls" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="config" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,22 +28,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E4057"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -58,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,12 +418,9 @@
   </sheetPr>
   <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
@@ -442,35 +429,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Oatly</t>
+          <t>Alpha Foods</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Beta Beverages</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Califia</t>
+          <t>Gamma Nutrition</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Silk</t>
+          <t>Delta Farms</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Elmhurst</t>
+          <t>Epsilon Brands</t>
         </is>
       </c>
     </row>
@@ -487,24 +474,19 @@
   </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="75" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>depth</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
@@ -513,7 +495,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.oatly.com/oatly-who/sustainability-plan/sustainability-report</t>
+          <t>https://www.alpha-foods.example/sustainability</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -521,14 +503,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Oatly</t>
+          <t>Alpha Foods</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://ripplefoods.com/pages/our-story</t>
+          <t>https://www.beta-beverages.example/about</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -536,14 +518,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Beta Beverages</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.califiafarms.com/sustainability</t>
+          <t>https://www.gamma-nutrition.example/impact</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -551,14 +533,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Califia</t>
+          <t>Gamma Nutrition</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://silk.com/about-us/sustainability/</t>
+          <t>https://www.delta-farms.example/news/earth</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -566,14 +548,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Silk</t>
+          <t>Delta Farms</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://elmhurst1925.com/blogs/news/elmhurst-earth-makes-us-sustainable</t>
+          <t>https://www.epsilon-brands.example/esg</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -581,14 +563,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Elmhurst</t>
+          <t>Epsilon Brands</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.mintel.com/food-and-drink/plant-based-milk</t>
+          <t>https://www.industry-report.example/market-overview</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -609,18 +591,14 @@
   </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="49" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>instructions</t>
         </is>
@@ -675,18 +653,14 @@
   </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>

</xml_diff>